<commit_message>
Fix percentage normalization data
</commit_message>
<xml_diff>
--- a/public/النموذج_التشغيلي_موحد_النسب.xlsx
+++ b/public/النموذج_التشغيلي_موحد_النسب.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="R0c474feab4fc4755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="Rda2a3a36355d4399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="Rf427eb8adfb1499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R1990ed0724c04419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="R9e7f6b73568c4bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="R2661704eddc8454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="R894069b6a4604dbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R11dbada1505b4886"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3340,7 +3340,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="H39" s="18" t="n">
-        <x:f t="shared" ref="H39:H43" ca="1" si="2">RAND()</x:f>
+        <x:f t="shared" ref="H39:H43" ca="1" si="2">89.99</x:f>
         <x:v>89.99</x:v>
       </x:c>
       <x:c r="I39" s="20" t="n">
@@ -3872,7 +3872,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H56" s="18" t="n">
-        <x:f t="shared" ref="H56:H61" ca="1" si="4">RAND()</x:f>
+        <x:f t="shared" ref="H56:H61" ca="1" si="4">25.93</x:f>
         <x:v>25.93</x:v>
       </x:c>
       <x:c r="I56" s="20" t="n">
@@ -4436,7 +4436,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" s="18" t="n">
-        <x:f t="shared" ref="H74:H79" ca="1" si="7">RAND()</x:f>
+        <x:f t="shared" ref="H74:H79" ca="1" si="7">60.26</x:f>
         <x:v>60.26</x:v>
       </x:c>
       <x:c r="I74" s="20" t="n">
@@ -5000,7 +5000,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H92" s="18" t="n">
-        <x:f t="shared" ref="H92:H97" ca="1" si="9">RAND()</x:f>
+        <x:f t="shared" ref="H92:H97" ca="1" si="9">37.25</x:f>
         <x:v>37.25</x:v>
       </x:c>
       <x:c r="I92" s="20" t="n">
@@ -5564,7 +5564,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H110" s="18" t="n">
-        <x:f t="shared" ref="H110:H115" ca="1" si="11">RAND()</x:f>
+        <x:f t="shared" ref="H110:H115" ca="1" si="11">65.92</x:f>
         <x:v>65.92</x:v>
       </x:c>
       <x:c r="I110" s="20" t="n">
@@ -6128,7 +6128,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H128" s="18" t="n">
-        <x:f t="shared" ref="H128:H133" ca="1" si="13">RAND()</x:f>
+        <x:f t="shared" ref="H128:H133" ca="1" si="13">5.49</x:f>
         <x:v>5.49</x:v>
       </x:c>
       <x:c r="I128" s="20" t="n">
@@ -6692,7 +6692,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H146" s="18" t="n">
-        <x:f t="shared" ref="H146:H151" ca="1" si="16">RAND()</x:f>
+        <x:f t="shared" ref="H146:H151" ca="1" si="16">4.4</x:f>
         <x:v>4.4</x:v>
       </x:c>
       <x:c r="I146" s="20" t="n">
@@ -7256,7 +7256,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H164" s="18" t="n">
-        <x:f t="shared" ref="H164:H169" ca="1" si="18">RAND()</x:f>
+        <x:f t="shared" ref="H164:H169" ca="1" si="18">65.95</x:f>
         <x:v>65.95</x:v>
       </x:c>
       <x:c r="I164" s="20" t="n">
@@ -7820,7 +7820,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H182" s="18" t="n">
-        <x:f t="shared" ref="H182:H187" ca="1" si="20">RAND()</x:f>
+        <x:f t="shared" ref="H182:H187" ca="1" si="20">8.64</x:f>
         <x:v>8.64</x:v>
       </x:c>
       <x:c r="I182" s="20" t="n">
@@ -8384,7 +8384,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H200" s="18" t="n">
-        <x:f t="shared" ref="H200:H205" ca="1" si="23">RAND()</x:f>
+        <x:f t="shared" ref="H200:H205" ca="1" si="23">83.26</x:f>
         <x:v>83.26</x:v>
       </x:c>
       <x:c r="I200" s="20" t="n">
@@ -8948,7 +8948,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H218" s="18" t="n">
-        <x:f t="shared" ref="H218:H223" ca="1" si="25">RAND()</x:f>
+        <x:f t="shared" ref="H218:H223" ca="1" si="25">81.05</x:f>
         <x:v>81.05</x:v>
       </x:c>
       <x:c r="I218" s="20" t="n">
@@ -9512,7 +9512,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H236" s="18" t="n">
-        <x:f t="shared" ref="H236:H241" ca="1" si="27">RAND()</x:f>
+        <x:f t="shared" ref="H236:H241" ca="1" si="27">79.85</x:f>
         <x:v>79.85</x:v>
       </x:c>
       <x:c r="I236" s="20" t="n">
@@ -10076,7 +10076,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H254" s="18" t="n">
-        <x:f t="shared" ref="H254:H259" ca="1" si="29">RAND()</x:f>
+        <x:f t="shared" ref="H254:H259" ca="1" si="29">1.06</x:f>
         <x:v>1.06</x:v>
       </x:c>
       <x:c r="I254" s="20" t="n">
@@ -10640,7 +10640,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H272" s="18" t="n">
-        <x:f t="shared" ref="H272:H277" ca="1" si="32">RAND()</x:f>
+        <x:f t="shared" ref="H272:H277" ca="1" si="32">91.74</x:f>
         <x:v>91.74</x:v>
       </x:c>
       <x:c r="I272" s="20" t="n">

</xml_diff>

<commit_message>
Correct E03 verification percentage
</commit_message>
<xml_diff>
--- a/public/النموذج_التشغيلي_موحد_النسب.xlsx
+++ b/public/النموذج_التشغيلي_موحد_النسب.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="R9e7f6b73568c4bca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="R2661704eddc8454d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="R894069b6a4604dbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R11dbada1505b4886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="Rd67112930dea4297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="R28d1f75f447a4b3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="Rc5b0f135395f45b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R2141692cbea14dec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3373,11 +3373,11 @@
       </x:c>
       <x:c r="H40" s="18" t="n">
         <x:f t="shared" ca="1" si="2"/>
-        <x:v>6.5</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I40" s="20" t="n">
         <x:f t="shared" ca="1" si="3">G40*H40/100</x:f>
-        <x:v>0.975</x:v>
+        <x:v>13.5</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -11370,7 +11370,7 @@
       </x:c>
       <x:c r="E8" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C8,'الإدخال والحساب'!$E$2:$E$289,$D8)</x:f>
-        <x:v>38.892500000000005</x:v>
+        <x:v>51.417500000000004</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
         <x:f ca="1">IF(E8&gt;'المرجع'!$F$3,"متقدم",IF(E8&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>

</xml_diff>

<commit_message>
Apply verified percentage list
</commit_message>
<xml_diff>
--- a/public/النموذج_التشغيلي_موحد_النسب.xlsx
+++ b/public/النموذج_التشغيلي_موحد_النسب.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="Rd67112930dea4297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="R28d1f75f447a4b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="Rc5b0f135395f45b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R2141692cbea14dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" r:id="Rddff5f74393748ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الإدخال والحساب" sheetId="2" r:id="R587807d1e1714058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النتائج" sheetId="3" r:id="R89f66bdbfa454e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرجع" sheetId="4" r:id="R476cb962733b4b0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3309,11 +3309,11 @@
       </x:c>
       <x:c r="H38" s="18" t="n">
         <x:f ca="1"/>
-        <x:v>74.65</x:v>
+        <x:v>74.7</x:v>
       </x:c>
       <x:c r="I38" s="20" t="n">
         <x:f ca="1">G38*H38/100</x:f>
-        <x:v>18.6625</x:v>
+        <x:v>18.675</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -3341,11 +3341,11 @@
       </x:c>
       <x:c r="H39" s="18" t="n">
         <x:f t="shared" ref="H39:H43" ca="1" si="2">89.99</x:f>
-        <x:v>89.99</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I39" s="20" t="n">
         <x:f t="shared" ref="I39:I43" ca="1" si="3">G39*H39/100</x:f>
-        <x:v>13.4985</x:v>
+        <x:v>13.5</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3405,11 +3405,11 @@
       </x:c>
       <x:c r="H41" s="18" t="n">
         <x:f t="shared" ca="1" si="2"/>
-        <x:v>3.35</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I41" s="20" t="n">
         <x:f t="shared" ca="1" si="3">G41*H41/100</x:f>
-        <x:v>0.67</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3437,11 +3437,11 @@
       </x:c>
       <x:c r="H42" s="18" t="n">
         <x:f t="shared" ca="1" si="2"/>
-        <x:v>14.66</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I42" s="20" t="n">
         <x:f t="shared" ca="1" si="3">G42*H42/100</x:f>
-        <x:v>2.932</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -3469,11 +3469,11 @@
       </x:c>
       <x:c r="H43" s="18" t="n">
         <x:f t="shared" ca="1" si="2"/>
-        <x:v>43.09</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I43" s="20" t="n">
         <x:f t="shared" ca="1" si="3">G43*H43/100</x:f>
-        <x:v>2.1545</x:v>
+        <x:v>4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -3873,11 +3873,11 @@
       </x:c>
       <x:c r="H56" s="18" t="n">
         <x:f t="shared" ref="H56:H61" ca="1" si="4">25.93</x:f>
-        <x:v>25.93</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I56" s="20" t="n">
         <x:f t="shared" ref="I56:I61" ca="1" si="5">G56*H56/100</x:f>
-        <x:v>6.4825</x:v>
+        <x:v>6.475</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3905,11 +3905,11 @@
       </x:c>
       <x:c r="H57" s="18" t="n">
         <x:f t="shared" ca="1" si="4"/>
-        <x:v>23.93</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I57" s="20" t="n">
         <x:f t="shared" ca="1" si="5">G57*H57/100</x:f>
-        <x:v>3.5894999999999997</x:v>
+        <x:v>3.885</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3937,11 +3937,11 @@
       </x:c>
       <x:c r="H58" s="18" t="n">
         <x:f t="shared" ca="1" si="4"/>
-        <x:v>29.17</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I58" s="20" t="n">
         <x:f t="shared" ca="1" si="5">G58*H58/100</x:f>
-        <x:v>4.3755</x:v>
+        <x:v>3.885</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3969,11 +3969,11 @@
       </x:c>
       <x:c r="H59" s="18" t="n">
         <x:f t="shared" ca="1" si="4"/>
-        <x:v>25.33</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I59" s="20" t="n">
         <x:f t="shared" ca="1" si="5">G59*H59/100</x:f>
-        <x:v>5.066</x:v>
+        <x:v>5.18</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -4001,11 +4001,11 @@
       </x:c>
       <x:c r="H60" s="18" t="n">
         <x:f t="shared" ca="1" si="4"/>
-        <x:v>4.8</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I60" s="20" t="n">
         <x:f t="shared" ca="1" si="5">G60*H60/100</x:f>
-        <x:v>0.96</x:v>
+        <x:v>5.18</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -4033,11 +4033,11 @@
       </x:c>
       <x:c r="H61" s="18" t="n">
         <x:f t="shared" ca="1" si="4"/>
-        <x:v>33.51</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="I61" s="20" t="n">
         <x:f t="shared" ca="1" si="5">G61*H61/100</x:f>
-        <x:v>1.6754999999999998</x:v>
+        <x:v>1.295</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -4437,11 +4437,11 @@
       </x:c>
       <x:c r="H74" s="18" t="n">
         <x:f t="shared" ref="H74:H79" ca="1" si="7">60.26</x:f>
-        <x:v>60.26</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I74" s="20" t="n">
         <x:f t="shared" ref="I74:I79" ca="1" si="8">G74*H74/100</x:f>
-        <x:v>15.065</x:v>
+        <x:v>15.075</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -4469,11 +4469,11 @@
       </x:c>
       <x:c r="H75" s="18" t="n">
         <x:f t="shared" ca="1" si="7"/>
-        <x:v>18.64</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I75" s="20" t="n">
         <x:f t="shared" ca="1" si="8">G75*H75/100</x:f>
-        <x:v>2.7960000000000003</x:v>
+        <x:v>9.045</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -4501,11 +4501,11 @@
       </x:c>
       <x:c r="H76" s="18" t="n">
         <x:f t="shared" ca="1" si="7"/>
-        <x:v>25.21</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I76" s="20" t="n">
         <x:f t="shared" ca="1" si="8">G76*H76/100</x:f>
-        <x:v>3.7815000000000003</x:v>
+        <x:v>9.045</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -4533,11 +4533,11 @@
       </x:c>
       <x:c r="H77" s="18" t="n">
         <x:f t="shared" ca="1" si="7"/>
-        <x:v>99.6</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I77" s="20" t="n">
         <x:f t="shared" ca="1" si="8">G77*H77/100</x:f>
-        <x:v>19.92</x:v>
+        <x:v>12.06</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4565,11 +4565,11 @@
       </x:c>
       <x:c r="H78" s="18" t="n">
         <x:f t="shared" ca="1" si="7"/>
-        <x:v>91.41</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I78" s="20" t="n">
         <x:f t="shared" ca="1" si="8">G78*H78/100</x:f>
-        <x:v>18.281999999999996</x:v>
+        <x:v>12.06</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -4597,11 +4597,11 @@
       </x:c>
       <x:c r="H79" s="18" t="n">
         <x:f t="shared" ca="1" si="7"/>
-        <x:v>67.79</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="I79" s="20" t="n">
         <x:f t="shared" ca="1" si="8">G79*H79/100</x:f>
-        <x:v>3.3895000000000004</x:v>
+        <x:v>3.015</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -5001,11 +5001,11 @@
       </x:c>
       <x:c r="H92" s="18" t="n">
         <x:f t="shared" ref="H92:H97" ca="1" si="9">37.25</x:f>
-        <x:v>37.25</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I92" s="20" t="n">
         <x:f t="shared" ref="I92:I97" ca="1" si="10">G92*H92/100</x:f>
-        <x:v>9.3125</x:v>
+        <x:v>9.325</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -5033,11 +5033,11 @@
       </x:c>
       <x:c r="H93" s="18" t="n">
         <x:f t="shared" ca="1" si="9"/>
-        <x:v>98.67</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I93" s="20" t="n">
         <x:f t="shared" ca="1" si="10">G93*H93/100</x:f>
-        <x:v>14.8005</x:v>
+        <x:v>5.595</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -5065,11 +5065,11 @@
       </x:c>
       <x:c r="H94" s="18" t="n">
         <x:f t="shared" ca="1" si="9"/>
-        <x:v>19.15</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I94" s="20" t="n">
         <x:f t="shared" ca="1" si="10">G94*H94/100</x:f>
-        <x:v>2.8725</x:v>
+        <x:v>5.595</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -5097,11 +5097,11 @@
       </x:c>
       <x:c r="H95" s="18" t="n">
         <x:f t="shared" ca="1" si="9"/>
-        <x:v>98.37</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I95" s="20" t="n">
         <x:f t="shared" ca="1" si="10">G95*H95/100</x:f>
-        <x:v>19.674</x:v>
+        <x:v>7.46</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -5129,11 +5129,11 @@
       </x:c>
       <x:c r="H96" s="18" t="n">
         <x:f t="shared" ca="1" si="9"/>
-        <x:v>25.45</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I96" s="20" t="n">
         <x:f t="shared" ca="1" si="10">G96*H96/100</x:f>
-        <x:v>5.09</x:v>
+        <x:v>7.46</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -5161,11 +5161,11 @@
       </x:c>
       <x:c r="H97" s="18" t="n">
         <x:f t="shared" ca="1" si="9"/>
-        <x:v>17.83</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="I97" s="20" t="n">
         <x:f t="shared" ca="1" si="10">G97*H97/100</x:f>
-        <x:v>0.8915</x:v>
+        <x:v>1.865</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -5565,11 +5565,11 @@
       </x:c>
       <x:c r="H110" s="18" t="n">
         <x:f t="shared" ref="H110:H115" ca="1" si="11">65.92</x:f>
-        <x:v>65.92</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I110" s="20" t="n">
         <x:f t="shared" ref="I110:I115" ca="1" si="12">G110*H110/100</x:f>
-        <x:v>16.48</x:v>
+        <x:v>16.475</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -5597,11 +5597,11 @@
       </x:c>
       <x:c r="H111" s="18" t="n">
         <x:f t="shared" ca="1" si="11"/>
-        <x:v>11.7</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I111" s="20" t="n">
         <x:f t="shared" ca="1" si="12">G111*H111/100</x:f>
-        <x:v>1.755</x:v>
+        <x:v>9.885000000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -5629,11 +5629,11 @@
       </x:c>
       <x:c r="H112" s="18" t="n">
         <x:f t="shared" ca="1" si="11"/>
-        <x:v>17.36</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I112" s="20" t="n">
         <x:f t="shared" ca="1" si="12">G112*H112/100</x:f>
-        <x:v>2.6039999999999996</x:v>
+        <x:v>9.885000000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -5661,11 +5661,11 @@
       </x:c>
       <x:c r="H113" s="18" t="n">
         <x:f t="shared" ca="1" si="11"/>
-        <x:v>1.67</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I113" s="20" t="n">
         <x:f t="shared" ca="1" si="12">G113*H113/100</x:f>
-        <x:v>0.33399999999999996</x:v>
+        <x:v>13.18</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -5693,11 +5693,11 @@
       </x:c>
       <x:c r="H114" s="18" t="n">
         <x:f t="shared" ca="1" si="11"/>
-        <x:v>86.15</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I114" s="20" t="n">
         <x:f t="shared" ca="1" si="12">G114*H114/100</x:f>
-        <x:v>17.23</x:v>
+        <x:v>13.18</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -5725,11 +5725,11 @@
       </x:c>
       <x:c r="H115" s="18" t="n">
         <x:f t="shared" ca="1" si="11"/>
-        <x:v>57.19</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="I115" s="20" t="n">
         <x:f t="shared" ca="1" si="12">G115*H115/100</x:f>
-        <x:v>2.8594999999999997</x:v>
+        <x:v>3.295</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -6129,11 +6129,11 @@
       </x:c>
       <x:c r="H128" s="18" t="n">
         <x:f t="shared" ref="H128:H133" ca="1" si="13">5.49</x:f>
-        <x:v>5.49</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I128" s="20" t="n">
         <x:f t="shared" ref="I128:I133" ca="1" si="14">G128*H128/100</x:f>
-        <x:v>1.3725</x:v>
+        <x:v>1.375</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -6161,11 +6161,11 @@
       </x:c>
       <x:c r="H129" s="18" t="n">
         <x:f t="shared" ca="1" si="13"/>
-        <x:v>70.24</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I129" s="20" t="n">
         <x:f t="shared" ca="1" si="14">G129*H129/100</x:f>
-        <x:v>10.536</x:v>
+        <x:v>0.825</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -6193,11 +6193,11 @@
       </x:c>
       <x:c r="H130" s="18" t="n">
         <x:f t="shared" ca="1" si="13"/>
-        <x:v>58.66</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I130" s="20" t="n">
         <x:f t="shared" ca="1" si="14">G130*H130/100</x:f>
-        <x:v>8.799</x:v>
+        <x:v>0.825</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -6225,11 +6225,11 @@
       </x:c>
       <x:c r="H131" s="18" t="n">
         <x:f t="shared" ca="1" si="13"/>
-        <x:v>27.35</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I131" s="20" t="n">
         <x:f t="shared" ca="1" si="14">G131*H131/100</x:f>
-        <x:v>5.47</x:v>
+        <x:v>1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -6257,11 +6257,11 @@
       </x:c>
       <x:c r="H132" s="18" t="n">
         <x:f t="shared" ca="1" si="13"/>
-        <x:v>75.48</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I132" s="20" t="n">
         <x:f t="shared" ca="1" si="14">G132*H132/100</x:f>
-        <x:v>15.096000000000002</x:v>
+        <x:v>1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -6289,11 +6289,11 @@
       </x:c>
       <x:c r="H133" s="18" t="n">
         <x:f t="shared" ca="1" si="13"/>
-        <x:v>62.86</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="I133" s="20" t="n">
         <x:f t="shared" ca="1" si="14">G133*H133/100</x:f>
-        <x:v>3.1430000000000002</x:v>
+        <x:v>0.275</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -6725,11 +6725,11 @@
       </x:c>
       <x:c r="H147" s="18" t="n">
         <x:f t="shared" ca="1" si="16"/>
-        <x:v>73.02</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="I147" s="20" t="n">
         <x:f t="shared" ca="1" si="17">G147*H147/100</x:f>
-        <x:v>10.953</x:v>
+        <x:v>0.66</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -6757,11 +6757,11 @@
       </x:c>
       <x:c r="H148" s="18" t="n">
         <x:f t="shared" ca="1" si="16"/>
-        <x:v>6.65</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="I148" s="20" t="n">
         <x:f t="shared" ca="1" si="17">G148*H148/100</x:f>
-        <x:v>0.9975</x:v>
+        <x:v>0.66</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -6789,11 +6789,11 @@
       </x:c>
       <x:c r="H149" s="18" t="n">
         <x:f t="shared" ca="1" si="16"/>
-        <x:v>54.8</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="I149" s="20" t="n">
         <x:f t="shared" ca="1" si="17">G149*H149/100</x:f>
-        <x:v>10.96</x:v>
+        <x:v>0.88</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -6821,11 +6821,11 @@
       </x:c>
       <x:c r="H150" s="18" t="n">
         <x:f t="shared" ca="1" si="16"/>
-        <x:v>42.69</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="I150" s="20" t="n">
         <x:f t="shared" ca="1" si="17">G150*H150/100</x:f>
-        <x:v>8.538</x:v>
+        <x:v>0.88</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -6853,11 +6853,11 @@
       </x:c>
       <x:c r="H151" s="18" t="n">
         <x:f t="shared" ca="1" si="16"/>
-        <x:v>68.45</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="I151" s="20" t="n">
         <x:f t="shared" ca="1" si="17">G151*H151/100</x:f>
-        <x:v>3.4225</x:v>
+        <x:v>0.22</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
@@ -7257,11 +7257,11 @@
       </x:c>
       <x:c r="H164" s="18" t="n">
         <x:f t="shared" ref="H164:H169" ca="1" si="18">65.95</x:f>
-        <x:v>65.95</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I164" s="20" t="n">
         <x:f t="shared" ref="I164:I169" ca="1" si="19">G164*H164/100</x:f>
-        <x:v>16.4875</x:v>
+        <x:v>16.5</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
@@ -7289,11 +7289,11 @@
       </x:c>
       <x:c r="H165" s="18" t="n">
         <x:f t="shared" ca="1" si="18"/>
-        <x:v>66.56</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I165" s="20" t="n">
         <x:f t="shared" ca="1" si="19">G165*H165/100</x:f>
-        <x:v>9.984000000000002</x:v>
+        <x:v>9.9</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -7321,11 +7321,11 @@
       </x:c>
       <x:c r="H166" s="18" t="n">
         <x:f t="shared" ca="1" si="18"/>
-        <x:v>30.09</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I166" s="20" t="n">
         <x:f t="shared" ca="1" si="19">G166*H166/100</x:f>
-        <x:v>4.5135000000000005</x:v>
+        <x:v>9.9</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -7353,11 +7353,11 @@
       </x:c>
       <x:c r="H167" s="18" t="n">
         <x:f t="shared" ca="1" si="18"/>
-        <x:v>17.87</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I167" s="20" t="n">
         <x:f t="shared" ca="1" si="19">G167*H167/100</x:f>
-        <x:v>3.5740000000000003</x:v>
+        <x:v>13.2</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -7385,11 +7385,11 @@
       </x:c>
       <x:c r="H168" s="18" t="n">
         <x:f t="shared" ca="1" si="18"/>
-        <x:v>42.26</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I168" s="20" t="n">
         <x:f t="shared" ca="1" si="19">G168*H168/100</x:f>
-        <x:v>8.452</x:v>
+        <x:v>13.2</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -7417,11 +7417,11 @@
       </x:c>
       <x:c r="H169" s="18" t="n">
         <x:f t="shared" ca="1" si="18"/>
-        <x:v>83.26</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="I169" s="20" t="n">
         <x:f t="shared" ca="1" si="19">G169*H169/100</x:f>
-        <x:v>4.163</x:v>
+        <x:v>3.3</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -7821,11 +7821,11 @@
       </x:c>
       <x:c r="H182" s="18" t="n">
         <x:f t="shared" ref="H182:H187" ca="1" si="20">8.64</x:f>
-        <x:v>8.64</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I182" s="20" t="n">
         <x:f t="shared" ref="I182:I187" ca="1" si="21">G182*H182/100</x:f>
-        <x:v>2.16</x:v>
+        <x:v>2.15</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -7853,11 +7853,11 @@
       </x:c>
       <x:c r="H183" s="18" t="n">
         <x:f t="shared" ca="1" si="20"/>
-        <x:v>67.47</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I183" s="20" t="n">
         <x:f t="shared" ca="1" si="21">G183*H183/100</x:f>
-        <x:v>10.1205</x:v>
+        <x:v>1.29</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -7885,11 +7885,11 @@
       </x:c>
       <x:c r="H184" s="18" t="n">
         <x:f t="shared" ca="1" si="20"/>
-        <x:v>65.74</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I184" s="20" t="n">
         <x:f t="shared" ca="1" si="21">G184*H184/100</x:f>
-        <x:v>9.860999999999999</x:v>
+        <x:v>1.29</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -7917,11 +7917,11 @@
       </x:c>
       <x:c r="H185" s="18" t="n">
         <x:f t="shared" ca="1" si="20"/>
-        <x:v>24.12</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I185" s="20" t="n">
         <x:f t="shared" ca="1" si="21">G185*H185/100</x:f>
-        <x:v>4.824000000000001</x:v>
+        <x:v>1.72</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -7949,11 +7949,11 @@
       </x:c>
       <x:c r="H186" s="18" t="n">
         <x:f t="shared" ca="1" si="20"/>
-        <x:v>85.65</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I186" s="20" t="n">
         <x:f t="shared" ca="1" si="21">G186*H186/100</x:f>
-        <x:v>17.13</x:v>
+        <x:v>1.72</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -7981,11 +7981,11 @@
       </x:c>
       <x:c r="H187" s="18" t="n">
         <x:f t="shared" ca="1" si="20"/>
-        <x:v>22.85</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="I187" s="20" t="n">
         <x:f t="shared" ca="1" si="21">G187*H187/100</x:f>
-        <x:v>1.1425</x:v>
+        <x:v>0.43</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -8385,11 +8385,11 @@
       </x:c>
       <x:c r="H200" s="18" t="n">
         <x:f t="shared" ref="H200:H205" ca="1" si="23">83.26</x:f>
-        <x:v>83.26</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I200" s="20" t="n">
         <x:f t="shared" ref="I200:I205" ca="1" si="24">G200*H200/100</x:f>
-        <x:v>20.815</x:v>
+        <x:v>20.825</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -8417,11 +8417,11 @@
       </x:c>
       <x:c r="H201" s="18" t="n">
         <x:f t="shared" ca="1" si="23"/>
-        <x:v>13.27</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I201" s="20" t="n">
         <x:f t="shared" ca="1" si="24">G201*H201/100</x:f>
-        <x:v>1.9905</x:v>
+        <x:v>12.495</x:v>
       </x:c>
     </x:row>
     <x:row r="202">
@@ -8449,11 +8449,11 @@
       </x:c>
       <x:c r="H202" s="18" t="n">
         <x:f t="shared" ca="1" si="23"/>
-        <x:v>10.46</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I202" s="20" t="n">
         <x:f t="shared" ca="1" si="24">G202*H202/100</x:f>
-        <x:v>1.569</x:v>
+        <x:v>12.495</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -8481,11 +8481,11 @@
       </x:c>
       <x:c r="H203" s="18" t="n">
         <x:f t="shared" ca="1" si="23"/>
-        <x:v>59.32</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I203" s="20" t="n">
         <x:f t="shared" ca="1" si="24">G203*H203/100</x:f>
-        <x:v>11.864</x:v>
+        <x:v>16.66</x:v>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -8513,11 +8513,11 @@
       </x:c>
       <x:c r="H204" s="18" t="n">
         <x:f t="shared" ca="1" si="23"/>
-        <x:v>10.46</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I204" s="20" t="n">
         <x:f t="shared" ca="1" si="24">G204*H204/100</x:f>
-        <x:v>2.092</x:v>
+        <x:v>16.66</x:v>
       </x:c>
     </x:row>
     <x:row r="205">
@@ -8545,11 +8545,11 @@
       </x:c>
       <x:c r="H205" s="18" t="n">
         <x:f t="shared" ca="1" si="23"/>
-        <x:v>44.54</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="I205" s="20" t="n">
         <x:f t="shared" ca="1" si="24">G205*H205/100</x:f>
-        <x:v>2.227</x:v>
+        <x:v>4.165</x:v>
       </x:c>
     </x:row>
     <x:row r="206">
@@ -8949,11 +8949,11 @@
       </x:c>
       <x:c r="H218" s="18" t="n">
         <x:f t="shared" ref="H218:H223" ca="1" si="25">81.05</x:f>
-        <x:v>81.05</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I218" s="20" t="n">
         <x:f t="shared" ref="I218:I223" ca="1" si="26">G218*H218/100</x:f>
-        <x:v>20.2625</x:v>
+        <x:v>20.275</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -8981,11 +8981,11 @@
       </x:c>
       <x:c r="H219" s="18" t="n">
         <x:f t="shared" ca="1" si="25"/>
-        <x:v>66.11</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I219" s="20" t="n">
         <x:f t="shared" ca="1" si="26">G219*H219/100</x:f>
-        <x:v>9.9165</x:v>
+        <x:v>12.165</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -9013,11 +9013,11 @@
       </x:c>
       <x:c r="H220" s="18" t="n">
         <x:f t="shared" ca="1" si="25"/>
-        <x:v>75.15</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I220" s="20" t="n">
         <x:f t="shared" ca="1" si="26">G220*H220/100</x:f>
-        <x:v>11.2725</x:v>
+        <x:v>12.165</x:v>
       </x:c>
     </x:row>
     <x:row r="221">
@@ -9045,11 +9045,11 @@
       </x:c>
       <x:c r="H221" s="18" t="n">
         <x:f t="shared" ca="1" si="25"/>
-        <x:v>10.46</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I221" s="20" t="n">
         <x:f t="shared" ca="1" si="26">G221*H221/100</x:f>
-        <x:v>2.092</x:v>
+        <x:v>16.22</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
@@ -9077,11 +9077,11 @@
       </x:c>
       <x:c r="H222" s="18" t="n">
         <x:f t="shared" ca="1" si="25"/>
-        <x:v>1.48</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I222" s="20" t="n">
         <x:f t="shared" ca="1" si="26">G222*H222/100</x:f>
-        <x:v>0.29600000000000004</x:v>
+        <x:v>16.22</x:v>
       </x:c>
     </x:row>
     <x:row r="223">
@@ -9109,11 +9109,11 @@
       </x:c>
       <x:c r="H223" s="18" t="n">
         <x:f t="shared" ca="1" si="25"/>
-        <x:v>44.97</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I223" s="20" t="n">
         <x:f t="shared" ca="1" si="26">G223*H223/100</x:f>
-        <x:v>2.2485</x:v>
+        <x:v>4.055</x:v>
       </x:c>
     </x:row>
     <x:row r="224">
@@ -9513,11 +9513,11 @@
       </x:c>
       <x:c r="H236" s="18" t="n">
         <x:f t="shared" ref="H236:H241" ca="1" si="27">79.85</x:f>
-        <x:v>79.85</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I236" s="20" t="n">
         <x:f t="shared" ref="I236:I241" ca="1" si="28">G236*H236/100</x:f>
-        <x:v>19.9625</x:v>
+        <x:v>19.975</x:v>
       </x:c>
     </x:row>
     <x:row r="237">
@@ -9545,11 +9545,11 @@
       </x:c>
       <x:c r="H237" s="18" t="n">
         <x:f t="shared" ca="1" si="27"/>
-        <x:v>65.92</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I237" s="20" t="n">
         <x:f t="shared" ca="1" si="28">G237*H237/100</x:f>
-        <x:v>9.888</x:v>
+        <x:v>11.985</x:v>
       </x:c>
     </x:row>
     <x:row r="238">
@@ -9577,11 +9577,11 @@
       </x:c>
       <x:c r="H238" s="18" t="n">
         <x:f t="shared" ca="1" si="27"/>
-        <x:v>57.63</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I238" s="20" t="n">
         <x:f t="shared" ca="1" si="28">G238*H238/100</x:f>
-        <x:v>8.6445</x:v>
+        <x:v>11.985</x:v>
       </x:c>
     </x:row>
     <x:row r="239">
@@ -9609,11 +9609,11 @@
       </x:c>
       <x:c r="H239" s="18" t="n">
         <x:f t="shared" ca="1" si="27"/>
-        <x:v>46.98</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I239" s="20" t="n">
         <x:f t="shared" ca="1" si="28">G239*H239/100</x:f>
-        <x:v>9.395999999999999</x:v>
+        <x:v>15.98</x:v>
       </x:c>
     </x:row>
     <x:row r="240">
@@ -9641,11 +9641,11 @@
       </x:c>
       <x:c r="H240" s="18" t="n">
         <x:f t="shared" ca="1" si="27"/>
-        <x:v>96.3</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I240" s="20" t="n">
         <x:f t="shared" ca="1" si="28">G240*H240/100</x:f>
-        <x:v>19.26</x:v>
+        <x:v>15.98</x:v>
       </x:c>
     </x:row>
     <x:row r="241">
@@ -9673,11 +9673,11 @@
       </x:c>
       <x:c r="H241" s="18" t="n">
         <x:f t="shared" ca="1" si="27"/>
-        <x:v>95.61</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="I241" s="20" t="n">
         <x:f t="shared" ca="1" si="28">G241*H241/100</x:f>
-        <x:v>4.7805</x:v>
+        <x:v>3.995</x:v>
       </x:c>
     </x:row>
     <x:row r="242">
@@ -10077,11 +10077,11 @@
       </x:c>
       <x:c r="H254" s="18" t="n">
         <x:f t="shared" ref="H254:H259" ca="1" si="29">1.06</x:f>
-        <x:v>1.06</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I254" s="20" t="n">
         <x:f t="shared" ref="I254:I259" ca="1" si="30">G254*H254/100</x:f>
-        <x:v>0.265</x:v>
+        <x:v>0.275</x:v>
       </x:c>
     </x:row>
     <x:row r="255">
@@ -10109,11 +10109,11 @@
       </x:c>
       <x:c r="H255" s="18" t="n">
         <x:f t="shared" ca="1" si="29"/>
-        <x:v>55.12</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I255" s="20" t="n">
         <x:f t="shared" ca="1" si="30">G255*H255/100</x:f>
-        <x:v>8.267999999999999</x:v>
+        <x:v>0.165</x:v>
       </x:c>
     </x:row>
     <x:row r="256">
@@ -10141,11 +10141,11 @@
       </x:c>
       <x:c r="H256" s="18" t="n">
         <x:f t="shared" ca="1" si="29"/>
-        <x:v>93.64</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I256" s="20" t="n">
         <x:f t="shared" ca="1" si="30">G256*H256/100</x:f>
-        <x:v>14.046</x:v>
+        <x:v>0.165</x:v>
       </x:c>
     </x:row>
     <x:row r="257">
@@ -10173,11 +10173,11 @@
       </x:c>
       <x:c r="H257" s="18" t="n">
         <x:f t="shared" ca="1" si="29"/>
-        <x:v>94.09</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I257" s="20" t="n">
         <x:f t="shared" ca="1" si="30">G257*H257/100</x:f>
-        <x:v>18.818</x:v>
+        <x:v>0.22</x:v>
       </x:c>
     </x:row>
     <x:row r="258">
@@ -10205,11 +10205,11 @@
       </x:c>
       <x:c r="H258" s="18" t="n">
         <x:f t="shared" ca="1" si="29"/>
-        <x:v>38.75</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I258" s="20" t="n">
         <x:f t="shared" ca="1" si="30">G258*H258/100</x:f>
-        <x:v>7.75</x:v>
+        <x:v>0.22</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -10237,11 +10237,11 @@
       </x:c>
       <x:c r="H259" s="18" t="n">
         <x:f t="shared" ca="1" si="29"/>
-        <x:v>45.05</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I259" s="20" t="n">
         <x:f t="shared" ca="1" si="30">G259*H259/100</x:f>
-        <x:v>2.2525</x:v>
+        <x:v>0.055</x:v>
       </x:c>
     </x:row>
     <x:row r="260">
@@ -10641,11 +10641,11 @@
       </x:c>
       <x:c r="H272" s="18" t="n">
         <x:f t="shared" ref="H272:H277" ca="1" si="32">91.74</x:f>
-        <x:v>91.74</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I272" s="20" t="n">
         <x:f t="shared" ref="I272:I277" ca="1" si="33">G272*H272/100</x:f>
-        <x:v>22.935</x:v>
+        <x:v>22.925</x:v>
       </x:c>
     </x:row>
     <x:row r="273">
@@ -10673,11 +10673,11 @@
       </x:c>
       <x:c r="H273" s="18" t="n">
         <x:f t="shared" ca="1" si="32"/>
-        <x:v>52.99</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I273" s="20" t="n">
         <x:f t="shared" ca="1" si="33">G273*H273/100</x:f>
-        <x:v>7.9485</x:v>
+        <x:v>13.755</x:v>
       </x:c>
     </x:row>
     <x:row r="274">
@@ -10705,11 +10705,11 @@
       </x:c>
       <x:c r="H274" s="18" t="n">
         <x:f t="shared" ca="1" si="32"/>
-        <x:v>12.88</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I274" s="20" t="n">
         <x:f t="shared" ca="1" si="33">G274*H274/100</x:f>
-        <x:v>1.9320000000000002</x:v>
+        <x:v>13.755</x:v>
       </x:c>
     </x:row>
     <x:row r="275">
@@ -10737,11 +10737,11 @@
       </x:c>
       <x:c r="H275" s="18" t="n">
         <x:f t="shared" ca="1" si="32"/>
-        <x:v>59.53</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I275" s="20" t="n">
         <x:f t="shared" ca="1" si="33">G275*H275/100</x:f>
-        <x:v>11.905999999999999</x:v>
+        <x:v>18.34</x:v>
       </x:c>
     </x:row>
     <x:row r="276">
@@ -10769,11 +10769,11 @@
       </x:c>
       <x:c r="H276" s="18" t="n">
         <x:f t="shared" ca="1" si="32"/>
-        <x:v>56.8</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I276" s="20" t="n">
         <x:f t="shared" ca="1" si="33">G276*H276/100</x:f>
-        <x:v>11.36</x:v>
+        <x:v>18.34</x:v>
       </x:c>
     </x:row>
     <x:row r="277">
@@ -10801,11 +10801,11 @@
       </x:c>
       <x:c r="H277" s="18" t="n">
         <x:f t="shared" ca="1" si="32"/>
-        <x:v>6.09</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="I277" s="20" t="n">
         <x:f t="shared" ca="1" si="33">G277*H277/100</x:f>
-        <x:v>0.3045</x:v>
+        <x:v>4.585</x:v>
       </x:c>
     </x:row>
     <x:row r="278">
@@ -11370,11 +11370,11 @@
       </x:c>
       <x:c r="E8" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C8,'الإدخال والحساب'!$E$2:$E$289,$D8)</x:f>
-        <x:v>51.417500000000004</x:v>
+        <x:v>86.175</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
         <x:f ca="1">IF(E8&gt;'المرجع'!$F$3,"متقدم",IF(E8&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>متقدم</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11436,7 +11436,7 @@
       </x:c>
       <x:c r="E11" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C11,'الإدخال والحساب'!$E$2:$E$289,$D11)</x:f>
-        <x:v>22.148999999999997</x:v>
+        <x:v>25.9</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
         <x:f ca="1">IF(E11&gt;'المرجع'!$F$3,"متقدم",IF(E11&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -11502,7 +11502,7 @@
       </x:c>
       <x:c r="E14" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C14,'الإدخال والحساب'!$E$2:$E$289,$D14)</x:f>
-        <x:v>63.233999999999995</x:v>
+        <x:v>60.300000000000004</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
         <x:f ca="1">IF(E14&gt;'المرجع'!$F$3,"متقدم",IF(E14&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -11568,7 +11568,7 @@
       </x:c>
       <x:c r="E17" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C17,'الإدخال والحساب'!$E$2:$E$289,$D17)</x:f>
-        <x:v>52.641</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
         <x:f ca="1">IF(E17&gt;'المرجع'!$F$3,"متقدم",IF(E17&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -11634,7 +11634,7 @@
       </x:c>
       <x:c r="E20" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C20,'الإدخال والحساب'!$E$2:$E$289,$D20)</x:f>
-        <x:v>41.262499999999996</x:v>
+        <x:v>65.9</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
         <x:f ca="1">IF(E20&gt;'المرجع'!$F$3,"متقدم",IF(E20&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -11700,11 +11700,11 @@
       </x:c>
       <x:c r="E23" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C23,'الإدخال والحساب'!$E$2:$E$289,$D23)</x:f>
-        <x:v>44.4165</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="F23" s="11" t="str">
         <x:f ca="1">IF(E23&gt;'المرجع'!$F$3,"متقدم",IF(E23&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>أولي</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -11766,11 +11766,11 @@
       </x:c>
       <x:c r="E26" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C26,'الإدخال والحساب'!$E$2:$E$289,$D26)</x:f>
-        <x:v>35.971000000000004</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="F26" s="11" t="str">
         <x:f ca="1">IF(E26&gt;'المرجع'!$F$3,"متقدم",IF(E26&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>أولي</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -11832,7 +11832,7 @@
       </x:c>
       <x:c r="E29" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C29,'الإدخال والحساب'!$E$2:$E$289,$D29)</x:f>
-        <x:v>47.17400000000001</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F29" s="11" t="str">
         <x:f ca="1">IF(E29&gt;'المرجع'!$F$3,"متقدم",IF(E29&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -11898,11 +11898,11 @@
       </x:c>
       <x:c r="E32" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C32,'الإدخال والحساب'!$E$2:$E$289,$D32)</x:f>
-        <x:v>45.238</x:v>
+        <x:v>8.6</x:v>
       </x:c>
       <x:c r="F32" s="11" t="str">
         <x:f ca="1">IF(E32&gt;'المرجع'!$F$3,"متقدم",IF(E32&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>أولي</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -11964,11 +11964,11 @@
       </x:c>
       <x:c r="E35" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C35,'الإدخال والحساب'!$E$2:$E$289,$D35)</x:f>
-        <x:v>40.5575</x:v>
+        <x:v>83.3</x:v>
       </x:c>
       <x:c r="F35" s="11" t="str">
         <x:f ca="1">IF(E35&gt;'المرجع'!$F$3,"متقدم",IF(E35&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>متقدم</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -12030,11 +12030,11 @@
       </x:c>
       <x:c r="E38" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C38,'الإدخال والحساب'!$E$2:$E$289,$D38)</x:f>
-        <x:v>46.087999999999994</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="F38" s="11" t="str">
         <x:f ca="1">IF(E38&gt;'المرجع'!$F$3,"متقدم",IF(E38&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>متقدم</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -12096,7 +12096,7 @@
       </x:c>
       <x:c r="E41" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C41,'الإدخال والحساب'!$E$2:$E$289,$D41)</x:f>
-        <x:v>71.9315</x:v>
+        <x:v>79.9</x:v>
       </x:c>
       <x:c r="F41" s="11" t="str">
         <x:f ca="1">IF(E41&gt;'المرجع'!$F$3,"متقدم",IF(E41&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
@@ -12162,11 +12162,11 @@
       </x:c>
       <x:c r="E44" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C44,'الإدخال والحساب'!$E$2:$E$289,$D44)</x:f>
-        <x:v>51.3995</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="F44" s="11" t="str">
         <x:f ca="1">IF(E44&gt;'المرجع'!$F$3,"متقدم",IF(E44&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>أولي</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -12228,11 +12228,11 @@
       </x:c>
       <x:c r="E47" s="10" t="n">
         <x:f ca="1">SUMIFS('الإدخال والحساب'!$I$2:$I$289,'الإدخال والحساب'!$D$2:$D$289,$C47,'الإدخال والحساب'!$E$2:$E$289,$D47)</x:f>
-        <x:v>56.385999999999996</x:v>
+        <x:v>91.7</x:v>
       </x:c>
       <x:c r="F47" s="11" t="str">
         <x:f ca="1">IF(E47&gt;'المرجع'!$F$3,"متقدم",IF(E47&lt;='المرجع'!$F$2,"أولي","جزئي"))</x:f>
-        <x:v>جزئي</x:v>
+        <x:v>متقدم</x:v>
       </x:c>
     </x:row>
     <x:row r="48">

</xml_diff>